<commit_message>
AIX 7.3 v8: add 11-special-features.md (5 feature articles, ~2400 lines), detail v7 S-rank config procedures (13 items, 100-200 lines each), neutralize qualitative descriptions. Maintains v6 commands+all-options 710 and v4-v7 11-section staple structure.
</commit_message>
<xml_diff>
--- a/docs/products/files/AIX_7.3.xlsx
+++ b/docs/products/files/AIX_7.3.xlsx
@@ -9,7 +9,7 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00_概要" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_コマンド" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01b_コマンド全オプション" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01b_コマンドオプション" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_設定値_tunable" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_設定値_file" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_用語集" sheetId="6" state="visible" r:id="rId6"/>
@@ -20,6 +20,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08_設定手順" sheetId="11" state="visible" r:id="rId11"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09_障害対応" sheetId="12" state="visible" r:id="rId12"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10_対象外項目" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11_特集記事" sheetId="14" state="visible" r:id="rId14"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -453,7 +454,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C20"/>
+  <dimension ref="A1:C21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -588,7 +589,7 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>hd5 = 40 MB（ディスク先頭 4GB 内、連続パーティション）</t>
+          <t>hd5 = 40 MB</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
@@ -639,7 +640,7 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>ksh（ksh88）/ ksh93 / bash（bash.rte）も TL3 で利用可</t>
+          <t>ksh（ksh88）/ ksh93 / bash</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
@@ -673,7 +674,7 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Python 3.9（python3.9.base） / 3.11（python3.11.base, 任意）</t>
+          <t>Python 3.9（python3.9.base）/ 3.11（任意）</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
@@ -707,7 +708,7 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>OpenSSL 3.0.x（TL3 SP1 = 3.0.15.1001）、OpenSSH 9.7p1</t>
+          <t>OpenSSL 3.0.x / OpenSSH 9.7p1</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
@@ -724,7 +725,7 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>45 件（v6 = 各コマンドに**全オプション** 710 件の日本語説明付き）</t>
+          <t>45 件 / 710 オプション</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
@@ -775,7 +776,7 @@
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>設定 18 / 障害対応 18（staple 15+ をカバー）</t>
+          <t>設定 18（うち S 級 13 件は詳細版）/ 障害対応 18</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
@@ -787,15 +788,32 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
+          <t>掲載特集記事</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>5 本（v8 新章、S 級ストーリー仕立て）</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>S_AIX73_review</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
           <t>ドキュメント形態</t>
         </is>
       </c>
-      <c r="B20" s="2" t="inlineStr">
+      <c r="B21" s="2" t="inlineStr">
         <is>
           <t>公式 IBM Docs Web + PDF（en/ja）</t>
         </is>
       </c>
-      <c r="C20" s="2" t="inlineStr">
+      <c r="C21" s="2" t="inlineStr">
         <is>
           <t>S_AIX73_install</t>
         </is>
@@ -5128,17 +5146,17 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>参照先（マニュアル名）</t>
+          <t>参照先</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>参照先 URL</t>
+          <t>URL</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>代表例（一部）</t>
+          <t>代表例</t>
         </is>
       </c>
     </row>
@@ -5732,6 +5750,210 @@
         <is>
           <t>メモリ ECC 多発; FC アダプタファームウェア不整合; Power FW のバグ起因の hang; PCI スロット不良; EPOW（Environmental and Power Warning）</t>
         </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <cols>
+    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="50" customWidth="1" min="2" max="2"/>
+    <col width="8" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="60" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>記事 ID</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>タイトル</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>重要度</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>カテゴリ</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>概要</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>本文行数</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>feature-01-disk-to-fs</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>ディスク容量確認から新規ファイルシステム作成まで</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>ストレージFS</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>ユーザから「データ置き場が欲しい」と依頼を受けて、既存容量を確認し、必要なら新規 PV を組み込んで LV/FS を作成、運用に引き渡すまでの一気通貫手順。</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="n">
+        <v>644</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>feature-02-perf-investigation</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>性能ボトルネック調査から改善・効果測定まで</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>性能</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>「業務系の応答が遅い」というクレームを受けて、CPU/メモリ/ディスク/ネットワークから真因を特定し、tunable や構成変更で改善、効果を定量測定して報告するまで。</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="n">
+        <v>413</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>feature-03-patch-apply</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>パッチ適用前準備から適用・検証・rollback まで</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>パッケージ</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>セキュリティ TL/SP 適用の標準手順。事前バックアップ → 適用 → 動作検証 → 失敗時の rollback まで。本番環境で安全に進めるためのチェックポイントを網羅。</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="n">
+        <v>534</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>feature-04-bulk-user-mgmt</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>ユーザ大量追加とグループ設計・監査ログ有効化</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>ユーザ認証</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>新部署発足や M&amp;A による 50 ユーザ一括追加。グループ設計、共通ポリシー適用、監査ログ有効化、定期棚卸しの仕組み構築まで。</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="n">
+        <v>548</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>feature-05-tcpip-change</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>TCP/IP 設定変更から検証・運用反映まで</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>ネットワーク</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>ネットワークセグメント変更（VLAN 移動・IP 帯変更）の本番系作業。事前準備から ifconfig 変更、ルーティング、DNS 更新、関連サーバ通知、業務確認まで。</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="n">
+        <v>341</v>
       </c>
     </row>
   </sheetData>
@@ -20181,7 +20403,7 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>影響範囲（applyType）</t>
+          <t>影響範囲</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
@@ -24205,7 +24427,7 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>errpt label / コード</t>
+          <t>errpt label</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">

</xml_diff>

<commit_message>
AIX 7.3 v9: 4 enhancements - glossary cross-links, playbook 22 cells detailed (~3000 lines), A-rank procedures detailed (config 5 + incident 6 = 11 items), 100+ diagrams extracted from official AIX manuals embedded in playbook/special-features/glossary/A-S detailed procedures.
</commit_message>
<xml_diff>
--- a/docs/products/files/AIX_7.3.xlsx
+++ b/docs/products/files/AIX_7.3.xlsx
@@ -9,7 +9,7 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00_概要" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_コマンド" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01b_コマンドオプション" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01b_オプション" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_設定値_tunable" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_設定値_file" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_用語集" sheetId="6" state="visible" r:id="rId6"/>
@@ -521,7 +521,7 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>AIX 7.3.4 / TL4（2025年12月リリース）</t>
+          <t>AIX 7.3.4 / TL4（2025年12月）</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
@@ -550,12 +550,12 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>最小メモリ要件</t>
+          <t>最小メモリ</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>4 GB（Quick Installation Guide v7.3 記載）</t>
+          <t>4 GB</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
@@ -567,12 +567,12 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>最小ディスク要件</t>
+          <t>最小ディスク</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>20 GB（既定 install）</t>
+          <t>20 GB</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
@@ -584,7 +584,7 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>ブートLV最小サイズ</t>
+          <t>ブートLV</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
@@ -606,7 +606,7 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>IBM Power Systems 上で稼働する 64-bit エンタープライズ UNIX OS</t>
+          <t>IBM Power Systems 上の 64-bit エンタープライズ UNIX OS</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
@@ -623,7 +623,7 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>AIX システム管理者、IBM Power サーバ運用者、UNIX 運用担当</t>
+          <t>AIX システム管理者</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
@@ -640,7 +640,7 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>ksh（ksh88）/ ksh93 / bash</t>
+          <t>ksh / bash</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
@@ -657,7 +657,7 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Java 8 64-bit（java8_64）</t>
+          <t>Java 8 64-bit</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
@@ -674,7 +674,7 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Python 3.9（python3.9.base）/ 3.11（任意）</t>
+          <t>Python 3.9 / 3.11</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
@@ -691,7 +691,7 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>SSHA-256（最大 255 文字）</t>
+          <t>SSHA-256</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
@@ -742,7 +742,7 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>40 件（tunable 20 + 設定ファイル 20）</t>
+          <t>40 件</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
@@ -759,7 +759,7 @@
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>65 件</t>
+          <t>65 件 (関連用語リンク化済み = v9)</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
@@ -776,7 +776,7 @@
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>設定 18（うち S 級 13 件は詳細版）/ 障害対応 18</t>
+          <t>設定 18 (S/A 詳細化) / 障害 18 (S/A 詳細化)</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
@@ -793,7 +793,7 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>5 本（v8 新章、S 級ストーリー仕立て）</t>
+          <t>5 本</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
@@ -805,17 +805,17 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>ドキュメント形態</t>
+          <t>プレイブック</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>公式 IBM Docs Web + PDF（en/ja）</t>
+          <t>22 セル (v9 で詳細化)</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>S_AIX73_install</t>
+          <t>S_AIX73_review</t>
         </is>
       </c>
     </row>
@@ -844,7 +844,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>出典 ID</t>
+          <t>ID</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
@@ -854,7 +854,7 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Form 番号</t>
+          <t>Form番号</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
@@ -5141,7 +5141,7 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>除外理由</t>
+          <t>理由</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
@@ -20408,7 +20408,7 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>関連パラメータ</t>
+          <t>関連</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
@@ -21403,7 +21403,7 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>編集者・コマンド</t>
+          <t>編集者</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
@@ -24164,221 +24164,752 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I4"/>
+  <dimension ref="A1:E23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="25" customWidth="1" min="2" max="2"/>
-    <col width="25" customWidth="1" min="3" max="3"/>
-    <col width="25" customWidth="1" min="4" max="4"/>
-    <col width="25" customWidth="1" min="5" max="5"/>
-    <col width="25" customWidth="1" min="6" max="6"/>
-    <col width="25" customWidth="1" min="7" max="7"/>
-    <col width="25" customWidth="1" min="8" max="8"/>
-    <col width="25" customWidth="1" min="9" max="9"/>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="40" customWidth="1" min="4" max="4"/>
+    <col width="60" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>習熟度＼シーン</t>
+          <t>習熟度</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
+          <t>シーン</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>タイトル</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>目的</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>ステップ要約</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>入門</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
           <t>構築</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>OS インストール → ホスト名/IP/DNS/NTP の基本設定</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>新規 LPAR を業務利用可能な最低限の状態まで構築する。</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>1. **インストール媒体から boot**
+   - HMC で LPAR を起動、SMS メニューで boot device 選択
+   - インストーラの「Default Install」または「Custom Install」を選択
+2. **基本ロケール・タイムゾーン設定**
+   - ロケール: ja_JP.UTF-8（または C）
+   - タイムゾーン: JST-9（日本時間）
+...</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>入門</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
         <is>
           <t>日常運用</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>errpt / df 定期チェック、syslog 設定</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>新人 AIX 管理者の日課 — エラー監視と容量監視。</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>1. **朝の errpt チェック**
+   - `errpt | head -20`（最新 20 件）
+   - `errpt -d H | head` （ハードウェアエラーのみ）
+   - 新規ハードエラーがあれば inc-errpt-hardware-error の手順へ
+2. **df で容量チェック**
+   - `df -g`（GB 単位で全 FS 表示）
+   - %Used 8...</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>入門</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
         <is>
           <t>バックアップ</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>mksysb で月次 rootvg バックアップ</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>DR 対策の最低限 — rootvg の bootable バックアップを定期取得。</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>1. **保管先空き確認**
+   - `df -g /backup`
+   - rootvg 実使用量の 1.5 倍以上推奨
+2. **mksysb 実行**
+   - `mksysb -i -X -e /backup/$(hostname)_$(date +%Y%m%d).mksysb`
+   - 数十分〜数時間（データ量による）
+3. **完了確認**
+   - 出力末尾: `0512-...</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>入門</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
         <is>
           <t>障害対応</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>boot 失敗・ログイン不可・FS full の三大障害</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>AIX 管理者が最初に覚える 3 つの基本障害対応。</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>1. **boot 失敗（LED hang）**
+   - HMC のオペレータパネルで LED コード記録
+   - SMS メニュー進入 → boot device 確認
+   - サービスモード boot → bosboot 再作成
+   - 詳細: [inc-boot-fail-led](09-incident-procedures.md#inc-boot-fail-led)
+2. **...</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>入門</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
         <is>
           <t>性能</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>topas / vmstat / iostat の読み方</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>性能監視の基本コマンド 3 つを使えるようになる。</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>1. **topas でリアルタイム概観**
+   - `topas`（5 秒間隔で更新）
+   - 画面の見方:
+     - 上部: CPU, Memory, Network, Disk のサマリ
+     - 中部: Network/Disk 統計
+     - 下部: プロセス一覧（CPU% 順）
+   - q で終了
+2. **vmstat で時系列観測**
+   - `vmstat ...</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>入門</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>セキュリティ</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>ユーザ追加とパスワードポリシー、SSH 鍵配置</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>セキュリティ運用の基本 — ユーザ管理と SSH 鍵認証。</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>1. **新規ユーザ追加**
+   - `mkuser id=2001 home=/home/alice shell=/usr/bin/ksh alice`
+   - 詳細: [cfg-user-add](08-config-procedures.md#cfg-user-add)
+2. **初期パスワード設定**
+   - `passwd alice`
+   - `pwdadm -f ADMCH...</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>中級</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>構築</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>VG/LV 設計、JFS2 FS 配置、rootvg ミラー化</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>業務系 LPAR の本格構築 — ストレージ設計と冗長化。</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>1. **新規 VG 設計と作成**
+   - 業務隔離するため datavg を新規作成
+   - `mkvg -S -y datavg -s 64 hdisk1`（scalable VG、PP=64MB）
+   - 詳細: [cfg-vg-lv](08-config-procedures.md#cfg-vg-lv)
+2. **業務 LV と FS の作成**
+   - DB データ用: `m...</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>中級</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>日常運用</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>errnotify でメール通知、cron 自動化、パッケージ更新管理</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>監視・通知の自動化と、パッケージ更新の管理ルーチン化。</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>1. **errnotify でメール通知設定**
+   - ハードエラー（Class=H）発生時に admin@example.com へ通知
+   - 詳細: [cfg-errnotify](08-config-procedures.md#cfg-errnotify)
+2. **cron で定期ジョブ登録**
+   - `crontab -e` で編集:
+   ```
+   # 朝 9 時に...</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>中級</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>バックアップ</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>mksysb + savevg、NIM image 連携</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>rootvg + 非 rootvg 両方のバックアップを取り、NIM 経由でリストア可能にする。</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>1. **rootvg バックアップ**
+   - `mksysb -i -X -e /backup/$(hostname)_rootvg_$(date +%Y%m%d).mksysb`
+   - 詳細: [cfg-mksysb-backup](08-config-procedures.md#cfg-mksysb-backup)
+2. **datavg バックアップ**
+   - `savevg...</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>中級</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>障害対応</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>性能低下切り分け、NFS stale、core 解析</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>中級レベルの障害切り分け — 複数仮説を立てて検証する手法。</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>1. **性能低下の切り分け**
+   - topas で CPU/Mem/Disk/Net の利用率を観察
+   - vmstat / iostat / netstat で詳細統計
+   - svmon -G でメモリ詳細
+   - 詳細: [inc-perf-degradation](09-incident-procedures.md#inc-perf-degradation)
+   - 特集...</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>中級</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>性能</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>TCP バッファ・MPIO queue_depth・j2_inodeCacheSize 調整</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>tunable 調整による性能改善。</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>1. **TCP 送受信バッファ拡大**
+   - 高遅延 WAN や 10GbE 環境で効果
+   - `no -p -o sb_max=4194304`
+   - `no -p -o tcp_sendspace=1048576`
+   - `no -p -o tcp_recvspace=1048576`
+   - 詳細: [cfg-tcp-buffers](08-config-procedur...</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>中級</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
         <is>
           <t>マイグレ</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>AIX 7.x → 7.3.4 マイグレ（premigration script、廃止 fileset）</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>旧 AIX バージョンから 7.3.4 への in-place マイグレーション。</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>1. **premigration script 実行**
+   - 旧版上で `/usr/lpp/bos/premig_chk` 実行
+   - チェック結果に従い廃止 fileset 削除等の準備
+2. **廃止 fileset の事前削除**
+   - `installp -u rsct.vsd` （VSD は AIX 7.3 で廃止）
+   - `installp -u rsct.lap...</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>中級</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
         <is>
           <t>セキュリティ</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>errnotify 監査連動、syslog 集中転送、LDAP クライアント</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>セキュリティ監視の集約化と、認証基盤統合。</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>1. **errnotify を監査ログに連動**
+   - errnotify で USER_LOCKED 等のセキュリティイベントを集中ログサーバへ転送
+   - 詳細: [cfg-errnotify](08-config-procedures.md#cfg-errnotify)
+2. **syslog 集中転送**
+   - `/etc/syslog.conf` に `*.info @lo...</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>中級</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
         <is>
           <t>スケーリング</t>
         </is>
       </c>
-    </row>
-    <row r="2" ht="90" customHeight="1">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>入門</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>OS インストール → ホスト名/IP/DNS/NTP の基本設定
-→ cfg-hostname-ip, cfg-dns, cfg-ntp</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>errpt / df 定期チェック、syslog 設定
-→ cfg-syslog, inc-fs-full</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>mksysb で月次 rootvg バックアップ
-→ cfg-mksysb-backup</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>boot 失敗・ログイン不可・FS full の三大障害
-→ inc-boot-fail-led, inc-login-locked, inc-fs-full</t>
-        </is>
-      </c>
-      <c r="F2" s="2" t="inlineStr">
-        <is>
-          <t>topas / vmstat / iostat の読み方
-→ inc-perf-degradation</t>
-        </is>
-      </c>
-      <c r="G2" s="2" t="inlineStr">
-        <is>
-          <t>（推奨せず — 上級者と協同）</t>
-        </is>
-      </c>
-      <c r="H2" s="2" t="inlineStr">
-        <is>
-          <t>ユーザ追加とパスワードポリシー、SSH 鍵配置
-→ cfg-user-add, cfg-passwd-policy</t>
-        </is>
-      </c>
-      <c r="I2" s="2" t="inlineStr">
-        <is>
-          <t>（推奨せず — 中級以降）</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="90" customHeight="1">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>中級</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>VG/LV 設計、JFS2 FS 配置、rootvg ミラー化
-→ cfg-vg-lv, cfg-rootvg-mirror</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>errnotify でメール通知、cron 自動化、パッケージ更新管理
-→ cfg-errnotify, cfg-package-install, inc-cron-fail</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>mksysb + savevg、NIM image 連携
-→ cfg-mksysb-backup</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
-          <t>性能低下切り分け（CPU/Mem/Disk/Net）、NFS stale、core 解析
-→ inc-perf-degradation, inc-nfs-stale, inc-core-dump</t>
-        </is>
-      </c>
-      <c r="F3" s="2" t="inlineStr">
-        <is>
-          <t>TCP バッファ・MPIO queue_depth・j2_inodeCacheSize 調整
-→ cfg-tcp-buffers, cfg-mpio-tuning, cfg-ioo-tuning</t>
-        </is>
-      </c>
-      <c r="G3" s="2" t="inlineStr">
-        <is>
-          <t>AIX 7.x → 7.3.4 マイグレ（premigration script、廃止 fileset）</t>
-        </is>
-      </c>
-      <c r="H3" s="2" t="inlineStr">
-        <is>
-          <t>errnotify 監査連動、syslog 集中転送、LDAP クライアント
-→ cfg-errnotify, cfg-syslog</t>
-        </is>
-      </c>
-      <c r="I3" s="2" t="inlineStr">
-        <is>
-          <t>FS 拡張、PV 追加、新規 VG 作成
-→ cfg-fs-extend, cfg-disk-add, cfg-vg-lv</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="90" customHeight="1">
-      <c r="A4" s="2" t="inlineStr">
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>FS 拡張、PV 追加、新規 VG 作成</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>業務拡大に伴うストレージ追加と容量拡張。</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>1. **新規 PV の認識**
+   - `cfgmgr -v` で新 hdisk 認識
+   - `lspv` で hdisk2 等が現れる
+   - PVID 付与: `chdev -l hdisk2 -a pv=yes`
+   - 詳細: [cfg-disk-add](08-config-procedures.md#cfg-disk-add)
+2. **既存 VG への追加**
+   -...</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
         <is>
           <t>上級</t>
         </is>
       </c>
-      <c r="B4" s="2" t="inlineStr">
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>構築</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
         <is>
           <t>NIM サーバ、CAA リポジトリ、PowerHA 連携、暗号化 rootvg</t>
         </is>
       </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>snap でサポート用情報定期取得、性能ベースライン取得（nmon）
-→ inc-snap-collect</t>
-        </is>
-      </c>
-      <c r="D4" s="2" t="inlineStr">
-        <is>
-          <t>NIM 連携の bootable mksysb、別 LPAR への restore リハーサル
-→ cfg-mksysb-backup</t>
-        </is>
-      </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
-          <t>kdb / dbx でカーネル / プロセスダンプ解析、HMC SRC コード解析
-→ inc-core-dump, inc-errpt-hardware-error</t>
-        </is>
-      </c>
-      <c r="F4" s="2" t="inlineStr">
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>高可用・大規模環境の基盤構築 — 上級者向けの専門手順群。</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>1. **NIM サーバ構築**
+   - bos.sysmgt.nim.master fileset 導入
+   - LPP_SOURCE 作成（base media + 必要 update を統合）
+   - SPOT 作成（ramdisk/カーネルイメージ）
+   - クライアント定義
+   - `nim -o define -t standalone -a platform=chrp .....</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>上級</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>日常運用</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>snap でサポート用情報定期取得、性能ベースライン取得（nmon）</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>上級運用の日課 — IBM サポート対応とトレンド分析の準備。</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>1. **月次 snap 取得**
+   - `snap -r` で旧データクリア
+   - `snap -ac` で全情報取得
+   - `/tmp/ibmsupt/snap.pax.gz` を IBM ECurep アップロード（PMR がある場合）
+   - 詳細: [inc-snap-collect](09-incident-procedures.md#inc-snap-collect)
+...</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>上級</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>バックアップ</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>NIM 連携の bootable mksysb、別 LPAR への restore リハーサル</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>DR 演習による実証 — mksysb から bootable restore できることを毎月確認。</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>1. **mksysb 取得（本番）**
+   - 詳細: [cfg-mksysb-backup](08-config-procedures.md#cfg-mksysb-backup)
+2. **NIM resource として登録**
+   - NIM サーバ側で:
+   - `nim -o define -t mksysb -a server=master -a location=... m...</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>上級</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>障害対応</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>kdb / dbx でカーネル / プロセスダンプ解析、HMC SRC コード解析</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>上級レベルの障害解析 — カーネルダンプとハードウェア診断。</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>1. **カーネルダンプ取得確認**
+   - `sysdumpdev -l` で primary が /dev/dumplv であること
+   - 詳細: [cfg-dump-device](08-config-procedures.md#cfg-dump-device)
+2. **kdb でカーネルダンプ解析**
+   - `kdb /var/adm/ras/vmcore.0`
+   - `...</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>上級</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>性能</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
         <is>
           <t>ASO/DSO 利用、large page 適用、AIO チューニング、NUMA awareness</t>
         </is>
       </c>
-      <c r="G4" s="2" t="inlineStr">
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>上級性能チューニング — ハードウェア特性を活かした最適化。</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>1. **ASO/DSO 有効化**
+   - Active System Optimizer / Dynamic System Optimizer
+   - `lssrc -s aso` で状態確認
+   - 起動: `startsrc -s aso`
+   - 自動最適化（large page、prefetch）
+2. **large page（16MB pages）適用**
+   - `v...</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>上級</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>セキュリティ</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>RBAC 設計、Trusted Execution + CHKSHOBJS、AIX Key Manager (PKS)、IPsec</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>上級セキュリティ — fine-grained 権限制御と暗号化機能。</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>1. **RBAC 設計**
+   - 業務別 role 定義: `mkrole authorizations=aix.network.config.* netadmin`
+   - ユーザに role 割当: `chuser roles=netadmin alice`
+   - swrole で role 切替: `swrole netadmin`
+2. **Domain RBAC（追加機能）...</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>上級</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>マイグレ</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
         <is>
           <t>Live Kernel Update、Live Library Update、別 LPAR への nimadm migration</t>
         </is>
       </c>
-      <c r="H4" s="2" t="inlineStr">
-        <is>
-          <t>RBAC 設計、Trusted Execution + CHKSHOBJS、AIX Key Manager (PKS)、IPsec</t>
-        </is>
-      </c>
-      <c r="I4" s="2" t="inlineStr">
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>業務無停止でのカーネル/ライブラリ更新と、別 LPAR への migration。</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>1. **Live Kernel Update (LKU)**
+   - 業務無停止でカーネル更新
+   - 互換性確認（TL/SP）
+   - `vi /etc/lvupdate.data`（ipsec_auto_migrate=yes 等）
+   - `geninstall` (LKU mode) または HMC ベース LKU
+   - blackout 時間中、アプリは一時停止
+   - ...</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>上級</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>スケーリング</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
         <is>
           <t>DLPAR でリソース動的増減、LPM で別物理機へ移動、scalable VG（1024 PV）</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>PowerVM 基盤を活かした動的スケーリング。</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>1. **DLPAR でメモリ追加**
+   - HMC でメモリ +XGB を実行
+   - AIX 側で `prtconf -m` で認識確認
+   - vmo tunable 見直し（minperm/maxperm 等）
+2. **DLPAR で CPU 追加**
+   - HMC で entitled processor units 増加
+   - AIX 側で `lparstat` で...</t>
         </is>
       </c>
     </row>
@@ -25115,7 +25646,7 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>参照章・観点</t>
+          <t>参照章</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">

</xml_diff>